<commit_message>
iteration2: finalize irr adjudication closeout
</commit_message>
<xml_diff>
--- a/data/labels/v1/irr_adjudication_sheet.xlsx
+++ b/data/labels/v1/irr_adjudication_sheet.xlsx
@@ -601,7 +601,11 @@
           <t>A-&gt;I</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -685,7 +689,11 @@
           <t>A-&gt;I</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
@@ -769,7 +777,11 @@
           <t>A-&gt;S</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
       <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -853,7 +865,11 @@
           <t>A-&gt;S</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -937,7 +953,11 @@
           <t>A-&gt;S</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1021,7 +1041,11 @@
           <t>A-&gt;I</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1105,7 +1129,11 @@
           <t>A-&gt;I</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -1189,7 +1217,11 @@
           <t>A-&gt;S</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
       <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1273,7 +1305,11 @@
           <t>A-&gt;I</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1357,7 +1393,11 @@
           <t>A-&gt;S</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1441,7 +1481,11 @@
           <t>A-&gt;I</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1525,7 +1569,11 @@
           <t>A-&gt;I</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1609,7 +1657,11 @@
           <t>S-&gt;I</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1693,7 +1745,11 @@
           <t>S-&gt;I</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1777,7 +1833,11 @@
           <t>S-&gt;I</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1861,7 +1921,11 @@
           <t>S-&gt;I</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
       <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1945,7 +2009,11 @@
           <t>S-&gt;A</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
       <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -2029,7 +2097,11 @@
           <t>S-&gt;I</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
       <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -2113,7 +2185,11 @@
           <t>S-&gt;A</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
       <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -2197,7 +2273,11 @@
           <t>S-&gt;A</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
       <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
@@ -2281,7 +2361,11 @@
           <t>S-&gt;A</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
       <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -2365,7 +2449,11 @@
           <t>S-&gt;I</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2449,7 +2537,11 @@
           <t>S-&gt;A</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
       <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
@@ -2533,7 +2625,11 @@
           <t>S-&gt;A</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Speculative</t>
+        </is>
+      </c>
       <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -2617,7 +2713,11 @@
           <t>S-&gt;I</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Irrelevant</t>
+        </is>
+      </c>
       <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -2701,7 +2801,11 @@
           <t>A-&gt;S</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Actionable</t>
+        </is>
+      </c>
       <c r="R27" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>